<commit_message>
Update data source and db file
</commit_message>
<xml_diff>
--- a/data/DLT历史数据_适配模型版.xlsx
+++ b/data/DLT历史数据_适配模型版.xlsx
@@ -358,7 +358,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2872"/>
+  <dimension ref="A1:H2873"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -75049,6 +75049,32 @@
         <v>9</v>
       </c>
     </row>
+    <row r="2873">
+      <c r="A2873" t="n">
+        <v>26054</v>
+      </c>
+      <c r="B2873" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2873" t="n">
+        <v>6</v>
+      </c>
+      <c r="D2873" t="n">
+        <v>14</v>
+      </c>
+      <c r="E2873" t="n">
+        <v>22</v>
+      </c>
+      <c r="F2873" t="n">
+        <v>24</v>
+      </c>
+      <c r="G2873" t="n">
+        <v>8</v>
+      </c>
+      <c r="H2873" t="n">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Add cross-period pattern recognition to the pool algorithm
</commit_message>
<xml_diff>
--- a/data/DLT历史数据_适配模型版.xlsx
+++ b/data/DLT历史数据_适配模型版.xlsx
@@ -358,7 +358,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2873"/>
+  <dimension ref="A1:H2874"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -75075,6 +75075,32 @@
         <v>11</v>
       </c>
     </row>
+    <row r="2874">
+      <c r="A2874" t="n">
+        <v>26055</v>
+      </c>
+      <c r="B2874" t="n">
+        <v>9</v>
+      </c>
+      <c r="C2874" t="n">
+        <v>10</v>
+      </c>
+      <c r="D2874" t="n">
+        <v>20</v>
+      </c>
+      <c r="E2874" t="n">
+        <v>33</v>
+      </c>
+      <c r="F2874" t="n">
+        <v>35</v>
+      </c>
+      <c r="G2874" t="n">
+        <v>4</v>
+      </c>
+      <c r="H2874" t="n">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 500.com as a backup source
</commit_message>
<xml_diff>
--- a/data/DLT历史数据_适配模型版.xlsx
+++ b/data/DLT历史数据_适配模型版.xlsx
@@ -358,7 +358,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2874"/>
+  <dimension ref="A1:H2875"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -75101,6 +75101,32 @@
         <v>11</v>
       </c>
     </row>
+    <row r="2875">
+      <c r="A2875" t="n">
+        <v>26056</v>
+      </c>
+      <c r="B2875" t="n">
+        <v>6</v>
+      </c>
+      <c r="C2875" t="n">
+        <v>7</v>
+      </c>
+      <c r="D2875" t="n">
+        <v>18</v>
+      </c>
+      <c r="E2875" t="n">
+        <v>21</v>
+      </c>
+      <c r="F2875" t="n">
+        <v>30</v>
+      </c>
+      <c r="G2875" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2875" t="n">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>

</xml_diff>